<commit_message>
Updates to align data files
</commit_message>
<xml_diff>
--- a/_readme/datafiles-draft.xlsx
+++ b/_readme/datafiles-draft.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -452,7 +452,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>./data/confidential/Jira Export CSV (my defaults) 20250218210036.csv</t>
+          <t>./data/crdcn-Publications-Export-2025-February-11-0901.csv</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>./data/confidential/jira-search-84765891-47e0-43ec-874d-365f527ef997.xlsx</t>
+          <t>./data/crossref_dois_enhanced.Rds</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -486,7 +486,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>./data/confidential/readme.txt</t>
+          <t>./data/crossref_dois.Rds</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -503,7 +503,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>./data/crdcn-Publications-Export-2025-February-11-0901.csv</t>
+          <t>./data/interwrk/cran_logs/2025-02-01-r.csv.gz</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -520,7 +520,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>./data/crossref_dois_enhanced.Rds</t>
+          <t>./data/interwrk/cran_logs/2025-02-02-r.csv.gz</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -537,7 +537,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>./data/crossref_dois.Rds</t>
+          <t>./data/interwrk/cran_logs/2025-02-03-r.csv.gz</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -554,7 +554,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-01-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-04-r.csv.gz</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -571,7 +571,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-02-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-05-r.csv.gz</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -588,7 +588,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-03-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-06-r.csv.gz</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -605,7 +605,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-04-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-07-r.csv.gz</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-05-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-08-r.csv.gz</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-06-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-09-r.csv.gz</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -656,7 +656,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-07-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-10-r.csv.gz</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -673,7 +673,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-08-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-11-r.csv.gz</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -690,7 +690,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-09-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-12-r.csv.gz</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-10-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-13-r.csv.gz</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -724,7 +724,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-11-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-14-r.csv.gz</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -741,7 +741,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-12-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-15-r.csv.gz</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-13-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-16-r.csv.gz</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-14-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-17-r.csv.gz</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -792,7 +792,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-15-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-18-r.csv.gz</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -809,7 +809,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-16-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-19-r.csv.gz</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -826,7 +826,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-17-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-20-r.csv.gz</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -843,7 +843,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-18-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-21-r.csv.gz</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -860,7 +860,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-19-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-22-r.csv.gz</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -877,7 +877,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-20-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-23-r.csv.gz</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -894,7 +894,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-21-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-24-r.csv.gz</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -911,7 +911,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-22-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-25-r.csv.gz</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -928,7 +928,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-23-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-26-r.csv.gz</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -945,7 +945,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-24-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-27-r.csv.gz</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -962,7 +962,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-25-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-02-28-r.csv.gz</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-26-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/2025-03-01-r.csv.gz</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -996,7 +996,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-27-r.csv.gz</t>
+          <t>./data/interwrk/cran_logs/downloaded_files_select.rds</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1013,7 +1013,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-02-28-r.csv.gz</t>
+          <t>./data/interwrk/r_downloads_by_country_select_nochina.csv</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1030,7 +1030,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/2025-03-01-r.csv.gz</t>
+          <t>./data/interwrk/r_downloads_by_country_select_nochina.rds</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1047,7 +1047,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>./data/interwrk/cran_logs/downloaded_files_select.rds</t>
+          <t>./data/interwrk/r_downloads_by_country_select.csv</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1064,7 +1064,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>./data/interwrk/geolocations.rds</t>
+          <t>./data/interwrk/r_downloads_by_country_select.rds</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_country_select_nochina.csv</t>
+          <t>./data/interwrk/r_downloads_by_global_select_nochina.csv</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1098,7 +1098,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_country_select_nochina.rds</t>
+          <t>./data/interwrk/r_downloads_by_global_select_nochina.rds</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1115,7 +1115,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_country_select.csv</t>
+          <t>./data/interwrk/r_downloads_by_global_select.csv</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1132,7 +1132,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_country_select.rds</t>
+          <t>./data/interwrk/r_downloads_by_global_select.rds</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1149,7 +1149,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_global_select_nochina.csv</t>
+          <t>./data/interwrk/r_downloads_by_region_select_nochina.csv</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1166,7 +1166,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_global_select_nochina.rds</t>
+          <t>./data/interwrk/r_downloads_by_region_select_nochina.rds</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_global_select.csv</t>
+          <t>./data/interwrk/r_downloads_by_region_select.csv</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1200,7 +1200,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_global_select.rds</t>
+          <t>./data/interwrk/r_downloads_by_region_select.rds</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_region_select_nochina.csv</t>
+          <t>./data/interwrk/r_downloads_select_combined.csv</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1234,7 +1234,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_region_select_nochina.rds</t>
+          <t>./data/interwrk/r_downloads_select_combined.rds</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1251,7 +1251,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_region_select.csv</t>
+          <t>./data/interwrk/stata_downloads_by_country_select_nochina.csv</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1268,7 +1268,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_by_region_select.rds</t>
+          <t>./data/interwrk/stata_downloads_by_country_select_nochina.rds</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_select_combined.csv</t>
+          <t>./data/interwrk/stata_downloads_by_country_select.csv</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1302,7 +1302,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>./data/interwrk/r_downloads_select_combined.rds</t>
+          <t>./data/interwrk/stata_downloads_by_country_select.rds</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1319,7 +1319,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>./data/interwrk/ssclogs.parquet</t>
+          <t>./data/interwrk/stata_downloads_by_global_select_nochina.csv</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1336,7 +1336,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>./data/interwrk/ssclogs.rds</t>
+          <t>./data/interwrk/stata_downloads_by_global_select_nochina.rds</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_country_select_nochina.csv</t>
+          <t>./data/interwrk/stata_downloads_by_global_select.csv</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_country_select_nochina.rds</t>
+          <t>./data/interwrk/stata_downloads_by_global_select.rds</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1387,7 +1387,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_country_select.csv</t>
+          <t>./data/interwrk/stata_downloads_by_region_select_nochina.csv</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1404,7 +1404,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_country_select.rds</t>
+          <t>./data/interwrk/stata_downloads_by_region_select_nochina.rds</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1421,7 +1421,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_global_select_nochina.csv</t>
+          <t>./data/interwrk/stata_downloads_by_region_select.csv</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1438,7 +1438,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_global_select_nochina.rds</t>
+          <t>./data/interwrk/stata_downloads_by_region_select.rds</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1455,7 +1455,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_global_select.csv</t>
+          <t>./data/issns.Rds</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1472,7 +1472,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_global_select.rds</t>
+          <t>./data/jira_access_cleaned.csv</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1489,7 +1489,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_region_select_nochina.csv</t>
+          <t>./data/jira_access_cleaned.Rds</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1506,7 +1506,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_region_select_nochina.rds</t>
+          <t>./data/nsf24336-tab001-005.xlsx</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1523,7 +1523,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_region_select.csv</t>
+          <t>./data/ProjectsAllMetadata_25JUN2024.xlsx</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1540,7 +1540,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>./data/interwrk/stata_downloads_by_region_select.rds</t>
+          <t>./data/PSID Bibliography Search.pdf</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1557,7 +1557,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>./data/issns.Rds</t>
+          <t>./data/restrictions.xlsx</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1574,7 +1574,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>./data/jira_access_cleaned.csv</t>
+          <t>./data/Screenshot 2025-02-08 at 19-49-29 PSID Bibliography Search.png</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1591,7 +1591,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>./data/jira_access_cleaned.Rds</t>
+          <t>./data/Screenshot 2025-05-16 at 14-49-46 CASD - Centre d'accès[...].png</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1608,7 +1608,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>./data/nsf24336-tab001-005.xlsx</t>
+          <t>./data/signal-2025-06-27-10-20-09-831.jpg</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1625,7 +1625,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>./data/ProjectsAllMetadata_25JUN2024.xlsx</t>
+          <t>./data/sources.txt</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1642,7 +1642,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>./data/PSID Bibliography Search.pdf</t>
+          <t>./data/stata-licenses-by-country.xlsx</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1651,125 +1651,6 @@
         </is>
       </c>
       <c r="D76" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>./data/raw/WebSTAR.log.gz</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>./data/restrictions.xlsx</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>./data/Screenshot 2025-02-08 at 19-49-29 PSID Bibliography Search.png</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>./data/Screenshot 2025-05-16 at 14-49-46 CASD - Centre d'accès[...].png</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>./data/signal-2025-06-27-10-20-09-831.jpg</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>./data/sources.txt</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>./data/stata-licenses-by-country.xlsx</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>